<commit_message>
feat: integrate logo, pre-production 0-entry baseline, and GitHub Pages/Vercel deployment
</commit_message>
<xml_diff>
--- a/Aerosol_Job_Card.xlsx
+++ b/Aerosol_Job_Card.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Aerosol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6806DB8D-CA41-4FD8-9138-C3340740DB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F681DF-13C2-499E-B4F2-71D0608E374E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1999,6 +1999,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
@@ -5134,6 +5138,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">

</xml_diff>